<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-04 La route des chaussettes jaunes
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-04.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-04.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Après la pluie, Mila veut une route de sable pour son doudou gris. Le doudou reste au bout. Elle reprend seau, manteau et doudou pour finir la route avec les chaussettes jaunes.</t>
+          <t>Le radiateur du couloir fait clic. Un éclat de lessive blanc brille sur une chaussette jaune. Mila veut la route jaune pour le doudou, maintenant. Au square, elle verse tout le sable d'un coup : la route s'effondre. Elle court avec le doudou seul, glisse, revient. Pelle, manteau, doudou. À la maison, elle tire les chaussettes d'un coup : tout tombe. Elle refuse de foncer. L'éclat penche vers la chaise. Elle pose, aligne, et l'éclat porte une trace de sable.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Près du radiateur, deux chaussettes jaunes sèchent. Elles sentent encore la lessive. Papa range les bottes mouillées. Une goutte tombe de la semelle. Tes chaussettes sont chaudes, Mila. Elles sont douces. On met les chaussettes sèches ? Mila enfile les chaussettes jaunes. Le radiateur fait un petit clic. On va au square ? Oui. Pour la route. Quelle route ? Pour le doudou. Ils ferment la porte. La rue sent la pluie. En ce moment, Mila est au square. Le sable est frais, encore un peu humide. Papa s'assoit près du bac. Mila a un seau jaune. Elle a un manteau bleu. Le doudou gris est au bout du bac. Le manteau est posé sur le banc. Je verse le sable, papa. Je t'écoute. Mila verse le sable. Ça fait chh. Le seau est froid contre ses mains. Un grain reste collé à son poignet. Il y a du sable sur toi. Sur le poignet. Mila fait une petite route. Le sable est frais sous les doigts. Ça sent la terre mouillée. Ça sent la pluie, encore. Oui, la pluie. Le doudou attend au bout de la route. Il va marcher. C'est l'heure. La route n'est pas finie. Le château de sable reste ici. La route, on la fera à la maison. On reprend ses affaires, avant de partir. Mila s'arrête. Le seau est encore dans le sable. Elle le prend. Le seau est là. Bien. Il servira pour la route. Le manteau est sur le banc. Le doudou est encore au bout. Un grain de sable est sur son nez.</t>
+          <t>Le radiateur du couloir fait clic. L'air tiède sent la laine mouillée. Sur une chaussette jaune, un éclat de lessive brille. Il est blanc, sec, et il pique un peu. Mila connaît ce couloir, ses dalles, ses bruits. Après la pluie, l'éclat paraît nouveau. Les bottes gouttent près de la porte. Je veux la route, maintenant ! Quelle route, Mila ? La route jaune, pour le doudou. On met les chaussettes ? Mila enfile la première, puis l'autre. L'éclat reste collé au fil. Elles sont chaudes ? Oui, papa. Ils ferment la porte. La rue sent la pluie et la terre. Une flaque brille entre deux dalles. En ce moment, Mila est au square. Le bac à sable luit, un peu sombre. Papa s'assoit près du bord. Le doudou gris attend au bout. Le manteau bleu repose sur le banc. Une pelle rouge est dans le sable. Je fais la route, tout de suite ! Je t'écoute. Mila verse tout le sable, d'un coup. Ça fait chh, trop fort. La route glisse et s'effondre. Le doudou tombe sur le flanc. Elle est cassée ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le sable a glissé ? Oui. Papa s'accroupit à la même hauteur. On peut en faire un bout. Mila tasse un petit chemin, lentement. Il peut marcher un peu. C'est l'heure. La route n'est pas finie. Mila saisit le doudou, rien d'autre. Elle court vers la grille. Le sable mouillé fait glisser le pied. Aïe ! La pelle reste dans le bac. Le manteau reste sur le banc. Mila s'arrête. Attends. Elle revient vers le bac. Elle prend la pelle rouge.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Près du radiateur, deux chaussettes jaunes sèchent. Elles sentent encore la lessive. Papa range les bottes mouillées. Une goutte tombe de la semelle. Tes chaussettes sont chaudes, Mila. Elles sont douces. On met les chaussettes sèches ? Mila enfile les chaussettes jaunes. Le radiateur fait un petit clic. On va au square ? Oui. Pour la route. Quelle route ? Pour le doudou. Ils ferment la porte. La rue sent la pluie. En ce moment, Mila est au square. Le sable est frais, encore un peu humide. Papa s'assoit près du bac. Mila a un seau jaune. Elle a un manteau bleu. Le doudou gris est au bout du bac. Le manteau est posé sur le banc. Je verse le sable, papa. Je t'écoute. Mila verse le sable. Ça fait chh. Le seau est froid contre ses mains. Un grain reste collé à son poignet. Il y a du sable sur toi. Sur le poignet. Mila fait une petite route. Le sable est frais sous les doigts. Ça sent la terre mouillée. Ça sent la pluie, encore. Oui, la pluie. Le doudou attend au bout de la route. Il va marcher. C'est l'heure. La route n'est pas finie. Le château de sable reste ici. La route, on la fera à la maison. On reprend ses affaires, avant de partir. Mila s'arrête. Le seau est encore dans le sable. Elle le prend. Le seau est là. Bien. Il servira pour la route. Le manteau est sur le banc. Le doudou est encore au bout. Un grain de sable est sur son nez.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le radiateur du couloir fait clic. L'air tiède sent la laine mouillée. Sur une chaussette jaune, un &lt;emphasis level="moderate"&gt;éclat de lessive&lt;/emphasis&gt; brille. Il est blanc, sec, et il pique un peu. Mila connaît ce couloir, ses dalles, ses bruits. Après la pluie, l'éclat paraît nouveau. Les bottes gouttent près de la porte. Je veux la route, maintenant ! Quelle route, Mila ? La route jaune, pour le doudou. On met les chaussettes ? Mila enfile la première, puis l'autre. L'éclat reste collé au fil. Elles sont chaudes ? Oui, papa. Ils ferment la porte. La rue sent la pluie et la terre. Une flaque brille entre deux dalles. En ce moment, Mila est au square. Le bac à sable luit, un peu sombre. Papa s'assoit près du bord. Le doudou gris attend au bout. Le manteau bleu repose sur le banc. Une pelle rouge est dans le sable. Je fais la route, tout de suite ! Je t'écoute. Mila verse tout le sable, d'un coup. Ça fait chh, trop fort. La route glisse et s'effondre. Le doudou tombe sur le flanc. Elle est cassée ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le sable a glissé ? Oui. Papa s'accroupit à la même hauteur. On peut en faire un bout. Mila tasse un petit chemin, lentement. Il peut marcher un peu. C'est l'heure. La route n'est pas finie. Mila saisit le doudou, rien d'autre. Elle court vers la grille. Le sable mouillé fait glisser le pied. Aïe ! La pelle reste dans le bac. Le manteau reste sur le banc. Mila s'arrête. Attends. Elle revient vers le bac. Elle prend la pelle rouge.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Théo joue au square, près de papa. Le sable est frais. Théo a un seau jaune. Il a un manteau bleu. Il a son doudou gris. Théo verse le sable. Ça fait chh. Papa dit : c'est l'heure. On va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires avant de partir. Théo cherche le seau. Il le prend. Théo cherche le manteau. Il le prend. Théo cherche le doudou. Il le prend. Ses affaires sont dans ses mains. Parce qu'il reprend ses affaires, ils peuvent partir. Papa dit : merci Théo. Tu as repris tes affaires avant de partir. Ils marchent vers la maison. Parce que le seau, le manteau et le doudou sont là, Théo est prêt. Papa tient le sac. Théo tient le doudou. [pause]</t>
+          <t>Le radiateur du couloir fait clic. L'air tiède sent la laine mouillée. Sur une chaussette jaune, un &lt;emphasis&gt;éclat de lessive&lt;/emphasis&gt; brille. Il est blanc, sec, et il pique un peu. Mila connaît ce couloir, ses dalles, ses bruits. Après la pluie, l'éclat paraît nouveau. Les bottes gouttent près de la porte. Je veux la route, maintenant ! Quelle route, Mila ? La route jaune, pour le doudou. On met les chaussettes ? Mila enfile la première, puis l'autre. L'éclat reste collé au fil. Elles sont chaudes ? Oui, papa. Ils ferment la porte. La rue sent la pluie et la terre. Une flaque brille entre deux dalles. En ce moment, Mila est au square. Le bac à sable luit, un peu sombre. Papa s'assoit près du bord. Le doudou gris attend au bout. Le manteau bleu repose sur le banc. Une pelle rouge est dans le sable. Je fais la route, tout de suite ! Je t'écoute. Mila verse tout le sable, d'un coup. Ça fait chh, trop fort. La route glisse et s'effondre. Le doudou tombe sur le flanc. Elle est cassée ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le sable a glissé ? Oui. Papa s'accroupit à la même hauteur. On peut en faire un bout. Mila tasse un petit chemin, lentement. Il peut marcher un peu. C'est l'heure. La route n'est pas finie. Mila saisit le doudou, rien d'autre. Elle court vers la grille. Le sable mouillé fait glisser le pied. Aïe ! La pelle reste dans le bac. Le manteau reste sur le banc. Mila s'arrête. Attends. Elle revient vers le bac. Elle prend la pelle rouge. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>éclat de lessive</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,66 +1326,69 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_route_jaune_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Près du radiateur, deux chaussettes jaunes sèchent.
-narrateur|Elles sentent encore la lessive.
-narrateur|Papa range les bottes mouillées.
-narrateur|Une goutte tombe de la semelle.
-papa|Tes chaussettes sont chaudes, Mila.
-enfant-f|Elles sont douces.
-papa|On met les chaussettes sèches ?
-narrateur|Mila enfile les chaussettes jaunes.
-narrateur|Le radiateur fait un petit clic.
-papa|On va au square ?
+          <t>narrateur|Le radiateur du couloir fait clic.
+narrateur|L'air tiède sent la laine mouillée.
+narrateur|Sur une chaussette jaune, un éclat de lessive brille.
+narrateur|Il est blanc, sec, et il pique un peu.
+narrateur|Mila connaît ce couloir, ses dalles, ses bruits.
+narrateur|Après la pluie, l'éclat paraît nouveau.
+narrateur|Les bottes gouttent près de la porte.
+enfant-f|Je veux la route, maintenant !
+papa|Quelle route, Mila ?
+enfant-f|La route jaune, pour le doudou.
+papa|On met les chaussettes ?
+narrateur|Mila enfile la première, puis l'autre.
+narrateur|L'éclat reste collé au fil.
+papa|Elles sont chaudes ?
+enfant-f|Oui, papa.
+narrateur|Ils ferment la porte.
+narrateur|La rue sent la pluie et la terre.
+narrateur|Une flaque brille entre deux dalles.
+narrateur|En ce moment, Mila est au square.
+narrateur|Le bac à sable luit, un peu sombre.
+narrateur|Papa s'assoit près du bord.
+narrateur|Le doudou gris attend au bout.
+narrateur|Le manteau bleu repose sur le banc.
+narrateur|Une pelle rouge est dans le sable.
+enfant-f|Je fais la route, tout de suite !
+papa|Je t'écoute.
+narrateur|Mila verse tout le sable, d'un coup.
+narrateur|Ça fait chh, trop fort.
+narrateur|La route glisse et s'effondre.
+narrateur|Le doudou tombe sur le flanc.
+enfant-f|Elle est cassée !
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Le sable a glissé ?
 enfant-f|Oui.
-enfant-f|Pour la route.
-papa|Quelle route ?
-enfant-f|Pour le doudou.
-narrateur|Ils ferment la porte.
-narrateur|La rue sent la pluie.
-narrateur|En ce moment, Mila est au square.
-narrateur|Le sable est frais, encore un peu humide.
-narrateur|Papa s'assoit près du bac.
-narrateur|Mila a un seau jaune.
-narrateur|Elle a un manteau bleu.
-narrateur|Le doudou gris est au bout du bac.
-narrateur|Le manteau est posé sur le banc.
-enfant-f|Je verse le sable, papa.
-papa|Je t'écoute.
-narrateur|Mila verse le sable.
-narrateur|Ça fait chh.
-narrateur|Le seau est froid contre ses mains.
-narrateur|Un grain reste collé à son poignet.
-papa|Il y a du sable sur toi.
-enfant-f|Sur le poignet.
-narrateur|Mila fait une petite route.
-narrateur|Le sable est frais sous les doigts.
-narrateur|Ça sent la terre mouillée.
-papa|Ça sent la pluie, encore.
-enfant-f|Oui, la pluie.
-narrateur|Le doudou attend au bout de la route.
-enfant-f|Il va marcher.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|On peut en faire un bout.
+narrateur|Mila tasse un petit chemin, lentement.
+enfant-f|Il peut marcher un peu.
 papa|C'est l'heure.
 enfant-f|La route n'est pas finie.
-papa|Le château de sable reste ici.
-papa|La route, on la fera à la maison.
-papa|On reprend ses affaires, avant de partir.
+narrateur|Mila saisit le doudou, rien d'autre.
+narrateur|Elle court vers la grille.
+narrateur|Le sable mouillé fait glisser le pied.
+enfant-f|Aïe !
+narrateur|La pelle reste dans le bac.
+narrateur|Le manteau reste sur le banc.
 narrateur|Mila s'arrête.
-narrateur|Le seau est encore dans le sable.
-narrateur|Elle le prend.
-enfant-f|Le seau est là.
-papa|Bien.
-papa|Il servira pour la route.
-narrateur|Le manteau est sur le banc.
-narrateur|Le doudou est encore au bout.
-narrateur|Un grain de sable est sur son nez.</t>
+enfant-f|Attends.
+narrateur|Elle revient vers le bac.
+narrateur|Elle prend la pelle rouge.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>radiateur,pluie,enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1412,17 +1415,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Mila ?</t>
+          <t>Mila tient la pelle. Avant de partir, que fait Mila ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Mila ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila tient la pelle. Avant de &lt;emphasis level="moderate"&gt;partir&lt;/emphasis&gt;, que fait Mila ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Théo ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila tient la pelle. Avant de &lt;emphasis&gt;partir&lt;/emphasis&gt;, que fait Mila ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1485,7 +1488,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1496,7 +1499,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1511,38 +1514,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>partir</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1557,22 +1560,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_partir_elle_prend_ses_affaires; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Mila ?</t>
+          <t>narrateur|Mila tient la pelle.
+narrateur|Avant de partir, que fait Mila ?</t>
         </is>
       </c>
     </row>
@@ -1599,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila cherche le manteau. Le tissu est un peu frais. Elle le prend. Le manteau aussi. Et le doudou ? Mila va au bout de la route. Elle essuie le grain sur le nez. Il est gris. Il est là. Elle le prend. Tu as repris tes affaires. Avant de partir. Oui. On peut continuer la route. Ils marchent vers la maison. Papa tient le sac. Mila tient le doudou. Tu es prête ? Je suis prête.</t>
+          <t>Mila cherche le manteau. Le tissu est un peu frais. Elle le prend. Le manteau aussi. Et le doudou ? Mila va au bout du bac. Le doudou a du sable sur l'oreille. Il est gris. Il est là. Elle le prend. Tu as la pelle ? Oui. On peut rentrer. Ils marchent vers la maison. La rue luit, un peu froide. Papa tient le sac. Mila tient le doudou. Tu es prête ? Je suis prête.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila cherche le manteau. Le tissu est un peu frais. Elle le prend. Le manteau aussi. Et le doudou ? Mila va au bout de la route. Elle essuie le grain sur le nez. Il est gris. Il est là. Elle le prend. Tu as repris tes affaires. Avant de partir. Oui. On peut continuer la route. Ils marchent vers la maison. Papa tient le sac. Mila tient le doudou. Tu es prête ? Je suis prête.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila cherche le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt;. Le tissu est un peu frais. Elle le prend. Le manteau aussi. Et le doudou ? Mila va au bout du bac. Le doudou a du sable sur l'oreille. Il est gris. Il est là. Elle le prend. Tu as la pelle ? Oui. On peut rentrer. Ils marchent vers la maison. La rue luit, un peu froide. Papa tient le sac. Mila tient le doudou. Tu es prête ? Je suis prête.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Théo a repris ses affaires. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. Papa est là. [pause]</t>
+          <t>Mila cherche le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Le tissu est un peu frais. Elle le prend. Le manteau aussi. Et le doudou ? Mila va au bout du bac. Le doudou a du sable sur l'oreille. Il est gris. Il est là. Elle le prend. Tu as la pelle ? Oui. On peut rentrer. Ils marchent vers la maison. La rue luit, un peu froide. Papa tient le sac. Mila tient le doudou. Tu es prête ? Je suis prête. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1667,7 +1671,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1690,11 +1694,11 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>manteau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>450</v>
@@ -1704,16 +1708,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1738,7 +1742,7 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=pelle_manteau_doudou_reviennent_avec_elle; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
@@ -1748,22 +1752,27 @@
 narrateur|Elle le prend.
 enfant-f|Le manteau aussi.
 papa|Et le doudou ?
-narrateur|Mila va au bout de la route.
-narrateur|Elle essuie le grain sur le nez.
+narrateur|Mila va au bout du bac.
+narrateur|Le doudou a du sable sur l'oreille.
 enfant-f|Il est gris.
 enfant-f|Il est là.
 narrateur|Elle le prend.
-papa|Tu as repris tes affaires.
-enfant-f|Avant de partir.
-papa|Oui.
-papa|On peut continuer la route.
+papa|Tu as la pelle ?
+enfant-f|Oui.
+papa|On peut rentrer.
 narrateur|Ils marchent vers la maison.
+narrateur|La rue luit, un peu froide.
 narrateur|Papa tient le sac.
 narrateur|Mila tient le doudou.
 papa|Tu es prête ?
 enfant-f|Je suis prête.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tissu,banc</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1788,17 +1797,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils arrivent à la porte. Les chaussettes jaunes ne sont plus au radiateur. Elles sont à tes pieds. Tu poses le seau près de la porte ? Mila pose le seau. Elle pose le manteau sur la chaise. Le doudou reste contre elle. On fait la route ici. Mila retire une chaussette jaune. Puis l'autre. Elle les pose en ligne sur le plancher. C'est la route. Le doudou peut marcher. Mila fait avancer le doudou. Pas à pas, sur le jaune. Il arrive. Bravo. Il a fini sa route. Le radiateur fait encore clic. La maison est tiède. Tu as les pieds au chaud, maintenant ? Oui, papa.</t>
+          <t>Ils arrivent à la porte. Les chaussettes jaunes ne sont plus au radiateur. Elles sont à tes pieds. La route, maintenant ! Mila tire les deux chaussettes, d'un coup. La pelle glisse entre ses bras. Le manteau tombe avec le doudou. Les chaussettes font un tas jaune. Elles se mélangent ! Mila refuse de foncer. Attends, je regarde. Personne ne dit le chemin. Mila écoute le couloir. Le radiateur chuchote. Sur la dalle, l'éclat de lessive tremble. Il penche vers la chaise. C'est là ! Mila pose la pelle près de la porte. Elle pose le manteau sur la chaise. Le doudou reste contre elle. Elle retire une chaussette, puis l'autre. Elle les pose en ligne sur le plancher. L'éclat revient sur le fil. C'est la route. Le doudou peut marcher. Mila fait avancer le doudou. Pas à pas, sur le jaune. Il arrive. Merci, Mila. On a fait la route ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils arrivent à la porte. Les chaussettes jaunes ne sont plus au radiateur. Elles sont à tes pieds. Tu poses le seau près de la porte ? Mila pose le seau. Elle pose le manteau sur la chaise. Le doudou reste contre elle. On fait la route ici. Mila retire une chaussette jaune. Puis l'autre. Elle les pose en ligne sur le plancher. C'est la route. Le doudou peut marcher. Mila fait avancer le doudou. Pas à pas, sur le jaune. Il arrive. Bravo. Il a fini sa route. Le radiateur fait encore clic. La maison est tiède. Tu as les pieds au chaud, maintenant ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils arrivent à la porte. Les chaussettes jaunes ne sont plus au radiateur. Elles sont à tes pieds. La route, maintenant ! Mila tire les deux chaussettes, d'un coup. La pelle glisse entre ses bras. Le manteau tombe avec le doudou. Les chaussettes font un tas jaune. Elles se mélangent ! Mila refuse de foncer. Attends, je regarde. Personne ne dit le chemin. Mila écoute le couloir. Le radiateur chuchote. Sur la dalle, l'&lt;emphasis level="moderate"&gt;éclat de lessive&lt;/emphasis&gt; tremble. Il penche vers la chaise. C'est là ! Mila pose la pelle près de la porte. Elle pose le manteau sur la chaise. Le doudou reste contre elle. Elle retire une chaussette, puis l'autre. Elle les pose en ligne sur le plancher. L'éclat revient sur le fil. C'est la route. Le doudou peut marcher. Mila fait avancer le doudou. Pas à pas, sur le jaune. Il arrive. Merci, Mila. On a fait la route ? Oui, papa.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Théo pose le seau près de la porte. Merci, dit papa. [pause]</t>
+          <t>Ils arrivent à la porte. Les chaussettes jaunes ne sont plus au radiateur. Elles sont à tes pieds. La route, maintenant ! Mila tire les deux chaussettes, d'un coup. La pelle glisse entre ses bras. Le manteau tombe avec le doudou. Les chaussettes font un tas jaune. Elles se mélangent ! Mila refuse de foncer. Attends, je regarde. Personne ne dit le chemin. Mila écoute le couloir. Le radiateur chuchote. Sur la dalle, l'&lt;emphasis&gt;éclat de lessive&lt;/emphasis&gt; tremble. Il penche vers la chaise. C'est là ! Mila pose la pelle près de la porte. Elle pose le manteau sur la chaise. Le doudou reste contre elle. Elle retire une chaussette, puis l'autre. Elle les pose en ligne sur le plancher. L'éclat revient sur le fil. C'est la route. Le doudou peut marcher. Mila fait avancer le doudou. Pas à pas, sur le jaune. Il arrive. Merci, Mila. On a fait la route ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1845,7 +1854,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1853,10 +1862,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1877,28 +1886,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de lessive</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1907,10 +1920,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1921,31 +1934,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_éclat_montre_la_chaise; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Ils arrivent à la porte.
 narrateur|Les chaussettes jaunes ne sont plus au radiateur.
 papa|Elles sont à tes pieds.
-papa|Tu poses le seau près de la porte ?
-narrateur|Mila pose le seau.
+enfant-f|La route, maintenant !
+narrateur|Mila tire les deux chaussettes, d'un coup.
+narrateur|La pelle glisse entre ses bras.
+narrateur|Le manteau tombe avec le doudou.
+narrateur|Les chaussettes font un tas jaune.
+enfant-f|Elles se mélangent !
+narrateur|Mila refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Personne ne dit le chemin.
+narrateur|Mila écoute le couloir.
+enfant-f|Le radiateur chuchote.
+narrateur|Sur la dalle, l'éclat de lessive tremble.
+narrateur|Il penche vers la chaise.
+enfant-f|C'est là !
+narrateur|Mila pose la pelle près de la porte.
 narrateur|Elle pose le manteau sur la chaise.
 narrateur|Le doudou reste contre elle.
-papa|On fait la route ici.
-narrateur|Mila retire une chaussette jaune.
-narrateur|Puis l'autre.
+narrateur|Elle retire une chaussette, puis l'autre.
 narrateur|Elle les pose en ligne sur le plancher.
+narrateur|L'éclat revient sur le fil.
 enfant-f|C'est la route.
 papa|Le doudou peut marcher.
 narrateur|Mila fait avancer le doudou.
 narrateur|Pas à pas, sur le jaune.
 enfant-f|Il arrive.
-papa|Bravo.
-papa|Il a fini sa route.
-narrateur|Le radiateur fait encore clic.
-narrateur|La maison est tiède.
-papa|Tu as les pieds au chaud, maintenant ?
+papa|Merci, Mila.
+papa|On a fait la route ?
 enfant-f|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>porte,radiateur,chaussettes</t>
         </is>
       </c>
     </row>
@@ -1972,17 +2003,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a fini sa route. Et toi, tu as repris tes affaires. Les chaussettes jaunes restent en ligne.</t>
+          <t>Le doudou s'arrête au bout du jaune. Mila pose les pieds sur le plancher tiède. Tes pieds sont au chaud ? Oui, papa. Le radiateur du couloir fait clic. L'éclat de lessive porte une trace de sable. Il a voyagé. Comme toi. Les chaussettes jaunes restent en ligne.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a fini sa route. Et toi, tu as repris tes affaires. Les chaussettes jaunes restent en ligne.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou s'arrête au bout du jaune. Mila pose les pieds sur le plancher tiède. Tes pieds sont au chaud ? Oui, papa. Le radiateur du couloir fait clic. L'&lt;emphasis level="moderate"&gt;éclat de lessive&lt;/emphasis&gt; porte une trace de sable. Il a voyagé. Comme toi. Les chaussettes jaunes restent en ligne.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou s'arrête au bout du jaune. Mila pose les pieds sur le plancher tiède. Tes pieds sont au chaud ? Oui, papa. Le radiateur du couloir fait clic. L'&lt;emphasis&gt;éclat de lessive&lt;/emphasis&gt; porte une trace de sable. Il a voyagé. Comme toi. Les chaussettes jaunes restent en ligne.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2029,7 +2060,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2037,10 +2068,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2049,12 +2080,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2063,17 +2094,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de lessive</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2082,11 +2117,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2095,26 +2130,41 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_porte_une_trace_de_sable; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Le doudou a fini sa route.
-papa|Et toi, tu as repris tes affaires.
+          <t>narrateur|Le doudou s'arrête au bout du jaune.
+narrateur|Mila pose les pieds sur le plancher tiède.
+papa|Tes pieds sont au chaud ?
+enfant-f|Oui, papa.
+narrateur|Le radiateur du couloir fait clic.
+narrateur|L'éclat de lessive porte une trace de sable.
+enfant-f|Il a voyagé.
+papa|Comme toi.
 narrateur|Les chaussettes jaunes restent en ligne.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur,plancher</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2227,6 +2277,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>